<commit_message>
correzione I e C
</commit_message>
<xml_diff>
--- a/questionari_sardi_outlier_sostituiti.xlsx
+++ b/questionari_sardi_outlier_sostituiti.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\salva\Desktop\Code\questionari2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D31488B-AB18-4687-8946-B290583AEBE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D437D83-B279-4706-BC98-743F082BFF4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9452,7 +9452,7 @@
         <v>79</v>
       </c>
       <c r="K17" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L17" t="s">
         <v>121</v>
@@ -12571,7 +12571,7 @@
         <v>76</v>
       </c>
       <c r="K51" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L51" t="s">
         <v>100</v>
@@ -22691,7 +22691,7 @@
         <v>79</v>
       </c>
       <c r="K167" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L167" t="s">
         <v>605</v>
@@ -23356,7 +23356,7 @@
         <v>79</v>
       </c>
       <c r="K177" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="L177" t="s">
         <v>619</v>
@@ -23734,7 +23734,7 @@
         <v>50</v>
       </c>
       <c r="K183" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L183" t="s">
         <v>549</v>
@@ -31156,7 +31156,7 @@
         <v>50</v>
       </c>
       <c r="K288" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L288" t="s">
         <v>85</v>
@@ -33324,7 +33324,7 @@
         <v>82</v>
       </c>
       <c r="K316" t="s">
-        <v>683</v>
+        <v>58</v>
       </c>
       <c r="L316" t="s">
         <v>183</v>
@@ -34327,7 +34327,7 @@
         <v>57</v>
       </c>
       <c r="K330" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="L330" t="s">
         <v>742</v>
@@ -39894,7 +39894,7 @@
         <v>79</v>
       </c>
       <c r="K400" t="s">
-        <v>683</v>
+        <v>58</v>
       </c>
       <c r="L400" t="s">
         <v>477</v>
@@ -43429,7 +43429,7 @@
         <v>76</v>
       </c>
       <c r="K453" t="s">
-        <v>683</v>
+        <v>73</v>
       </c>
       <c r="L453" t="s">
         <v>557</v>
@@ -45027,7 +45027,7 @@
         <v>79</v>
       </c>
       <c r="K478" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L478" t="s">
         <v>85</v>
@@ -46082,7 +46082,7 @@
         <v>130</v>
       </c>
       <c r="K494" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L494" t="s">
         <v>1266</v>
@@ -54075,7 +54075,7 @@
         <v>57</v>
       </c>
       <c r="K592" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="L592" t="s">
         <v>183</v>
@@ -54223,7 +54223,7 @@
         <v>79</v>
       </c>
       <c r="K594" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="L594" t="s">
         <v>183</v>
@@ -56525,7 +56525,7 @@
         <v>79</v>
       </c>
       <c r="K623" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L623" t="s">
         <v>1468</v>
@@ -62962,7 +62962,7 @@
         <v>79</v>
       </c>
       <c r="K705" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="L705" t="s">
         <v>522</v>

</xml_diff>